<commit_message>
Update base template and inject all 5 auto-calc formulas
Swapped in the newly attached 명세서(양식) file as the template. This
version has none of the calculated formulas prefilled (unlike the
previous upload, which had ③/⑧/⑫ but not ⑨/⑩) — so now injecting
all five: D10(③), D19(⑧), G8(⑨), G10(⑩), G15(⑫), matching the
formulas 사용안내 describes. Re-applied the D6 shrink-to-fit style
fix to this new template file as well.
</commit_message>
<xml_diff>
--- a/public/templates/resident-statement-template.xlsx
+++ b/public/templates/resident-statement-template.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\# 위드온빌리지\2_재무\입소비 청구\수급자 청구시스템\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53D05629-4FE9-4440-8B0B-BBC7404B0001}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21220" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="사용안내" sheetId="1" r:id="rId1"/>
@@ -1983,10 +1977,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="176" formatCode="0_);[Red]\(0\)"/>
+    <numFmt numFmtId="177" formatCode="#,##0_);[Red]\(#,##0\)"/>
   </numFmts>
   <fonts count="31">
     <font>
@@ -2478,9 +2472,6 @@
     <xf numFmtId="0" fontId="27" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="176" fontId="28" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2496,19 +2487,64 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2517,101 +2553,13 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="29" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="29" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="27" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2620,8 +2568,54 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="28" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="27" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="27" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="27" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="27" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="27" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="27" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="29" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="29" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2714,22 +2708,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>400050</xdr:colOff>
+      <xdr:colOff>240030</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>101600</xdr:rowOff>
+      <xdr:rowOff>53340</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>483281</xdr:colOff>
+      <xdr:colOff>498008</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>76881</xdr:rowOff>
+      <xdr:rowOff>206421</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="5" name="그림 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13C1A894-267A-4389-2F99-0D94AC03772B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{13C1A894-267A-4389-2F99-0D94AC03772B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2751,8 +2745,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5295900" y="8572500"/>
-          <a:ext cx="813481" cy="813481"/>
+          <a:off x="5040630" y="8519160"/>
+          <a:ext cx="974258" cy="991281"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2942,9 +2936,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="78" customWidth="1"/>
@@ -3055,43 +3049,43 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H27"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="18.5"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="18"/>
   <cols>
-    <col min="1" max="2" width="9.81640625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="15.90625" style="11" customWidth="1"/>
-    <col min="4" max="4" width="20.36328125" style="11" customWidth="1"/>
-    <col min="5" max="5" width="14.1796875" style="11" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" style="11" customWidth="1"/>
-    <col min="7" max="8" width="12.1796875" style="11" customWidth="1"/>
-    <col min="9" max="16384" width="8.6328125" style="11"/>
+    <col min="1" max="2" width="9.77734375" style="11" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" style="11" customWidth="1"/>
+    <col min="4" max="4" width="20.33203125" style="11" customWidth="1"/>
+    <col min="5" max="5" width="14.21875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" style="11" customWidth="1"/>
+    <col min="7" max="8" width="12.21875" style="11" customWidth="1"/>
+    <col min="9" max="16384" width="8.6640625" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20" customHeight="1">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:8" ht="19.95" customHeight="1">
+      <c r="A1" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
       <c r="G1" s="16"/>
       <c r="H1" s="18" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="20" customHeight="1">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
+    <row r="2" spans="1:8" ht="19.95" customHeight="1">
+      <c r="A2" s="53"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
       <c r="G2" s="17"/>
       <c r="H2" s="19" t="s">
         <v>97</v>
@@ -3101,292 +3095,283 @@
       <c r="A3" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="32"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="36"/>
       <c r="E3" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="30" t="s">
+      <c r="F3" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
     </row>
     <row r="4" spans="1:8" ht="33" customHeight="1">
       <c r="A4" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="32"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="36"/>
       <c r="E4" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
     </row>
     <row r="5" spans="1:8" ht="33" customHeight="1">
       <c r="A5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="B5" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="32"/>
+      <c r="C5" s="36"/>
       <c r="D5" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="40"/>
     </row>
     <row r="6" spans="1:8" ht="33" customHeight="1">
       <c r="A6" s="22"/>
-      <c r="B6" s="49"/>
-      <c r="C6" s="51"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="45"/>
       <c r="D6" s="23"/>
-      <c r="E6" s="49" t="s">
+      <c r="E6" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="44"/>
     </row>
     <row r="7" spans="1:8" ht="33" customHeight="1">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="31"/>
-      <c r="C7" s="32"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="36"/>
       <c r="D7" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="31"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="40"/>
     </row>
     <row r="8" spans="1:8" ht="33" customHeight="1">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="32"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="57" t="s">
+      <c r="C8" s="36"/>
+      <c r="D8" s="64"/>
+      <c r="E8" s="31" t="s">
         <v>89</v>
       </c>
-      <c r="F8" s="37"/>
-      <c r="G8" s="59"/>
-      <c r="H8" s="60"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="66"/>
     </row>
     <row r="9" spans="1:8" ht="33" customHeight="1">
-      <c r="A9" s="38"/>
-      <c r="B9" s="30" t="s">
+      <c r="A9" s="51"/>
+      <c r="B9" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="32"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="58"/>
-      <c r="F9" s="39"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="62"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="67"/>
+      <c r="H9" s="68"/>
     </row>
     <row r="10" spans="1:8" ht="33" customHeight="1">
-      <c r="A10" s="39"/>
-      <c r="B10" s="30" t="s">
+      <c r="A10" s="34"/>
+      <c r="B10" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="C10" s="32"/>
-      <c r="D10" s="24">
-        <f>D8+D9</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="30" t="s">
+      <c r="C10" s="36"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="F10" s="32"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="46"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="70"/>
     </row>
     <row r="11" spans="1:8" ht="33" customHeight="1">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="32"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="30" t="s">
+      <c r="C11" s="36"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="F11" s="32"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="46"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="70"/>
     </row>
     <row r="12" spans="1:8" ht="33" customHeight="1">
-      <c r="A12" s="38"/>
-      <c r="B12" s="30" t="s">
+      <c r="A12" s="51"/>
+      <c r="B12" s="35" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="32"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="40" t="s">
+      <c r="C12" s="36"/>
+      <c r="D12" s="64"/>
+      <c r="E12" s="37" t="s">
         <v>92</v>
       </c>
       <c r="F12" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="43"/>
-      <c r="H12" s="44"/>
+      <c r="G12" s="71"/>
+      <c r="H12" s="72"/>
     </row>
     <row r="13" spans="1:8" ht="33" customHeight="1">
-      <c r="A13" s="38"/>
-      <c r="B13" s="30" t="s">
+      <c r="A13" s="51"/>
+      <c r="B13" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="C13" s="32"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="41"/>
+      <c r="C13" s="36"/>
+      <c r="D13" s="64"/>
+      <c r="E13" s="38"/>
       <c r="F13" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="G13" s="43"/>
-      <c r="H13" s="44"/>
+      <c r="G13" s="71"/>
+      <c r="H13" s="72"/>
     </row>
     <row r="14" spans="1:8" ht="33" customHeight="1">
-      <c r="A14" s="38"/>
-      <c r="B14" s="40" t="s">
+      <c r="A14" s="51"/>
+      <c r="B14" s="37" t="s">
         <v>84</v>
       </c>
       <c r="C14" s="21"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="41"/>
+      <c r="D14" s="64"/>
+      <c r="E14" s="38"/>
       <c r="F14" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="43"/>
-      <c r="H14" s="44"/>
+      <c r="G14" s="71"/>
+      <c r="H14" s="72"/>
     </row>
     <row r="15" spans="1:8" ht="33" customHeight="1">
-      <c r="A15" s="38"/>
-      <c r="B15" s="41"/>
+      <c r="A15" s="51"/>
+      <c r="B15" s="38"/>
       <c r="C15" s="21"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="42"/>
+      <c r="D15" s="64"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="G15" s="45">
-        <f>G12+G13+G14</f>
-        <v>0</v>
-      </c>
-      <c r="H15" s="46"/>
+      <c r="G15" s="69"/>
+      <c r="H15" s="70"/>
     </row>
     <row r="16" spans="1:8" ht="33" customHeight="1">
-      <c r="A16" s="38"/>
-      <c r="B16" s="41"/>
+      <c r="A16" s="51"/>
+      <c r="B16" s="38"/>
       <c r="C16" s="21"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="30" t="s">
+      <c r="D16" s="64"/>
+      <c r="E16" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="40"/>
+      <c r="H16" s="40"/>
     </row>
     <row r="17" spans="1:8" ht="33" customHeight="1">
-      <c r="A17" s="38"/>
-      <c r="B17" s="41"/>
+      <c r="A17" s="51"/>
+      <c r="B17" s="38"/>
       <c r="C17" s="21"/>
-      <c r="D17" s="24"/>
+      <c r="D17" s="64"/>
       <c r="E17" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="30"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="40"/>
+      <c r="H17" s="40"/>
     </row>
     <row r="18" spans="1:8" ht="33" customHeight="1">
-      <c r="A18" s="38"/>
-      <c r="B18" s="42"/>
+      <c r="A18" s="51"/>
+      <c r="B18" s="39"/>
       <c r="C18" s="21"/>
-      <c r="D18" s="24"/>
+      <c r="D18" s="64"/>
       <c r="E18" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="F18" s="30"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="40"/>
+      <c r="H18" s="40"/>
     </row>
     <row r="19" spans="1:8" ht="33" customHeight="1">
-      <c r="A19" s="39"/>
-      <c r="B19" s="30" t="s">
+      <c r="A19" s="34"/>
+      <c r="B19" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="24">
-        <f>D11+D12+D13+SUM(D14:D18)</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="35" t="s">
+      <c r="C19" s="36"/>
+      <c r="D19" s="64"/>
+      <c r="E19" s="49" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
     </row>
     <row r="20" spans="1:8" ht="33" customHeight="1">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="55" t="s">
+      <c r="C20" s="27"/>
+      <c r="D20" s="29" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="56"/>
-      <c r="F20" s="28" t="s">
+      <c r="E20" s="30"/>
+      <c r="F20" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G20" s="25"/>
-      <c r="H20" s="29" t="s">
+      <c r="G20" s="24"/>
+      <c r="H20" s="28" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="33" customHeight="1">
-      <c r="A21" s="53"/>
-      <c r="B21" s="28" t="s">
+      <c r="A21" s="47"/>
+      <c r="B21" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="55" t="s">
+      <c r="C21" s="27"/>
+      <c r="D21" s="29" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="56"/>
-      <c r="F21" s="28" t="s">
+      <c r="E21" s="30"/>
+      <c r="F21" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="G21" s="26"/>
-      <c r="H21" s="27"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="26"/>
     </row>
     <row r="22" spans="1:8" ht="33" customHeight="1">
       <c r="A22" s="13">
@@ -3401,16 +3386,16 @@
       <c r="H22" s="15"/>
     </row>
     <row r="23" spans="1:8" ht="33" customHeight="1">
-      <c r="A23" s="54" t="s">
+      <c r="A23" s="48" t="s">
         <v>94</v>
       </c>
-      <c r="B23" s="54"/>
-      <c r="C23" s="54"/>
-      <c r="D23" s="54"/>
-      <c r="E23" s="54"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="54"/>
-      <c r="H23" s="54"/>
+      <c r="B23" s="48"/>
+      <c r="C23" s="48"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="48"/>
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="12"/>
@@ -3423,57 +3408,55 @@
       <c r="H24" s="12"/>
     </row>
     <row r="25" spans="1:8" ht="24" customHeight="1">
-      <c r="A25" s="47" t="s">
+      <c r="A25" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="47"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="47"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="47"/>
+      <c r="B25" s="41"/>
+      <c r="C25" s="41"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="41"/>
     </row>
     <row r="26" spans="1:8" ht="18" customHeight="1">
-      <c r="A26" s="47" t="s">
+      <c r="A26" s="41" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="47"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
+      <c r="B26" s="41"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="41"/>
+      <c r="H26" s="41"/>
     </row>
     <row r="27" spans="1:8" ht="18" customHeight="1">
-      <c r="A27" s="48" t="s">
+      <c r="A27" s="42" t="s">
         <v>88</v>
       </c>
-      <c r="B27" s="48"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="48"/>
-      <c r="H27" s="48"/>
+      <c r="B27" s="42"/>
+      <c r="C27" s="42"/>
+      <c r="D27" s="42"/>
+      <c r="E27" s="42"/>
+      <c r="F27" s="42"/>
+      <c r="G27" s="42"/>
+      <c r="H27" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="E8:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="E16:H16"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="G8:H9"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="A11:A19"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="E7:H7"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G15:H15"/>
     <mergeCell ref="A25:H25"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="A27:H27"/>
@@ -3490,19 +3473,21 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="A20:A21"/>
     <mergeCell ref="A23:H23"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="E8:F9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="E16:H16"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="G8:H9"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="F17:H17"/>
     <mergeCell ref="E19:H19"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A11:A19"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="F4:H4"/>
-    <mergeCell ref="A1:F2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -3513,12 +3498,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H33"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -3530,75 +3515,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="13.5" customHeight="1">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="62" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="G1" s="64" t="s">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="G1" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="H1" s="64"/>
+      <c r="H1" s="56"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="63" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="66" t="s">
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="57" t="s">
         <v>72</v>
       </c>
-      <c r="H2" s="66"/>
+      <c r="H2" s="57"/>
     </row>
     <row r="3" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A3" s="65"/>
-      <c r="B3" s="65"/>
-      <c r="C3" s="65"/>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
+      <c r="A3" s="63"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="63"/>
+      <c r="F3" s="63"/>
     </row>
     <row r="5" spans="1:8" ht="19.5" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="66" t="s">
+      <c r="B5" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="66"/>
-      <c r="D5" s="64" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="56" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="64"/>
-      <c r="F5" s="67" t="s">
+      <c r="E5" s="56"/>
+      <c r="F5" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
     </row>
     <row r="6" spans="1:8" ht="19.5" customHeight="1">
       <c r="A6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="67" t="s">
+      <c r="B6" s="59" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="67"/>
-      <c r="D6" s="64" t="s">
+      <c r="C6" s="59"/>
+      <c r="D6" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="64"/>
-      <c r="F6" s="66" t="s">
+      <c r="E6" s="56"/>
+      <c r="F6" s="57" t="s">
         <v>76</v>
       </c>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66"/>
+      <c r="G6" s="57"/>
+      <c r="H6" s="57"/>
     </row>
     <row r="7" spans="1:8" ht="19.5" customHeight="1">
       <c r="A7" s="5" t="s">
@@ -3607,16 +3592,16 @@
       <c r="B7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="64" t="s">
+      <c r="C7" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64" t="s">
+      <c r="D7" s="56"/>
+      <c r="E7" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
+      <c r="F7" s="56"/>
+      <c r="G7" s="56"/>
+      <c r="H7" s="56"/>
     </row>
     <row r="8" spans="1:8" ht="19.5" customHeight="1">
       <c r="A8" s="1" t="s">
@@ -3625,35 +3610,35 @@
       <c r="B8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="66" t="s">
+      <c r="C8" s="57" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="66"/>
-      <c r="E8" s="66" t="s">
+      <c r="D8" s="57"/>
+      <c r="E8" s="57" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="66"/>
-      <c r="G8" s="66"/>
-      <c r="H8" s="66"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="57"/>
+      <c r="H8" s="57"/>
     </row>
     <row r="9" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="64"/>
+      <c r="B9" s="56"/>
       <c r="C9" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="64" t="s">
+      <c r="D9" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="64"/>
-      <c r="F9" s="64"/>
-      <c r="G9" s="64"/>
-      <c r="H9" s="64"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
+      <c r="G9" s="56"/>
+      <c r="H9" s="56"/>
     </row>
     <row r="10" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A10" s="64" t="s">
+      <c r="A10" s="56" t="s">
         <v>35</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -3662,33 +3647,33 @@
       <c r="C10" s="2">
         <v>14800</v>
       </c>
-      <c r="D10" s="64" t="s">
+      <c r="D10" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="64"/>
-      <c r="F10" s="68">
+      <c r="E10" s="56"/>
+      <c r="F10" s="61">
         <f>C12+C23</f>
         <v>148000</v>
       </c>
-      <c r="G10" s="68"/>
-      <c r="H10" s="68"/>
+      <c r="G10" s="61"/>
+      <c r="H10" s="61"/>
     </row>
     <row r="11" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A11" s="64"/>
+      <c r="A11" s="56"/>
       <c r="B11" s="5" t="s">
         <v>38</v>
       </c>
       <c r="C11" s="2">
         <v>133200</v>
       </c>
-      <c r="D11" s="64"/>
-      <c r="E11" s="64"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="68"/>
-      <c r="H11" s="68"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
     </row>
     <row r="12" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A12" s="64"/>
+      <c r="A12" s="56"/>
       <c r="B12" s="5" t="s">
         <v>39</v>
       </c>
@@ -3696,19 +3681,19 @@
         <f>C10+C11</f>
         <v>148000</v>
       </c>
-      <c r="D12" s="64" t="s">
+      <c r="D12" s="56" t="s">
         <v>40</v>
       </c>
-      <c r="E12" s="64"/>
-      <c r="F12" s="68">
+      <c r="E12" s="56"/>
+      <c r="F12" s="61">
         <f>C10+C23</f>
         <v>14800</v>
       </c>
-      <c r="G12" s="68"/>
-      <c r="H12" s="68"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
     </row>
     <row r="13" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A13" s="64" t="s">
+      <c r="A13" s="56" t="s">
         <v>41</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -3717,170 +3702,170 @@
       <c r="C13" s="2">
         <v>0</v>
       </c>
-      <c r="D13" s="64"/>
-      <c r="E13" s="64"/>
-      <c r="F13" s="68"/>
-      <c r="G13" s="68"/>
-      <c r="H13" s="68"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
     </row>
     <row r="14" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A14" s="64"/>
+      <c r="A14" s="56"/>
       <c r="B14" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C14" s="2">
         <v>0</v>
       </c>
-      <c r="D14" s="64" t="s">
+      <c r="D14" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="64"/>
-      <c r="F14" s="69">
+      <c r="E14" s="56"/>
+      <c r="F14" s="60">
         <v>0</v>
       </c>
-      <c r="G14" s="69"/>
-      <c r="H14" s="69"/>
+      <c r="G14" s="60"/>
+      <c r="H14" s="60"/>
     </row>
     <row r="15" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A15" s="64"/>
+      <c r="A15" s="56"/>
       <c r="B15" s="5" t="s">
         <v>45</v>
       </c>
       <c r="C15" s="2">
         <v>0</v>
       </c>
-      <c r="D15" s="64"/>
-      <c r="E15" s="64"/>
-      <c r="F15" s="69"/>
-      <c r="G15" s="69"/>
-      <c r="H15" s="69"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="60"/>
+      <c r="G15" s="60"/>
+      <c r="H15" s="60"/>
     </row>
     <row r="16" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A16" s="64"/>
-      <c r="B16" s="64" t="s">
+      <c r="A16" s="56"/>
+      <c r="B16" s="56" t="s">
         <v>46</v>
       </c>
       <c r="C16" s="2">
         <v>0</v>
       </c>
-      <c r="D16" s="64" t="s">
+      <c r="D16" s="56" t="s">
         <v>47</v>
       </c>
-      <c r="E16" s="64"/>
+      <c r="E16" s="56"/>
       <c r="F16" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G16" s="69">
+      <c r="G16" s="60">
         <v>0</v>
       </c>
-      <c r="H16" s="69"/>
+      <c r="H16" s="60"/>
     </row>
     <row r="17" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A17" s="64"/>
-      <c r="B17" s="64"/>
+      <c r="A17" s="56"/>
+      <c r="B17" s="56"/>
       <c r="C17" s="2">
         <v>0</v>
       </c>
-      <c r="D17" s="64"/>
-      <c r="E17" s="64"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
       <c r="F17" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G17" s="69">
+      <c r="G17" s="60">
         <v>0</v>
       </c>
-      <c r="H17" s="69"/>
+      <c r="H17" s="60"/>
     </row>
     <row r="18" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A18" s="64"/>
-      <c r="B18" s="64"/>
+      <c r="A18" s="56"/>
+      <c r="B18" s="56"/>
       <c r="C18" s="2">
         <v>0</v>
       </c>
-      <c r="D18" s="64"/>
-      <c r="E18" s="64"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
       <c r="F18" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G18" s="69">
+      <c r="G18" s="60">
         <v>14800</v>
       </c>
-      <c r="H18" s="69"/>
+      <c r="H18" s="60"/>
     </row>
     <row r="19" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A19" s="64"/>
-      <c r="B19" s="64"/>
+      <c r="A19" s="56"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="2">
         <v>0</v>
       </c>
-      <c r="D19" s="64"/>
-      <c r="E19" s="64"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
       <c r="F19" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="68">
+      <c r="G19" s="61">
         <f>G16+G17+G18</f>
         <v>14800</v>
       </c>
-      <c r="H19" s="68"/>
+      <c r="H19" s="61"/>
     </row>
     <row r="20" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A20" s="64"/>
-      <c r="B20" s="64" t="s">
+      <c r="A20" s="56"/>
+      <c r="B20" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="68">
+      <c r="C20" s="61">
         <f>C13+C14+C15+SUM(C16:C19)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="64" t="s">
+      <c r="D20" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="64"/>
-      <c r="F20" s="64"/>
-      <c r="G20" s="64"/>
-      <c r="H20" s="64"/>
+      <c r="E20" s="56"/>
+      <c r="F20" s="56"/>
+      <c r="G20" s="56"/>
+      <c r="H20" s="56"/>
     </row>
     <row r="21" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A21" s="64"/>
-      <c r="B21" s="64"/>
-      <c r="C21" s="64"/>
-      <c r="D21" s="64" t="s">
+      <c r="A21" s="56"/>
+      <c r="B21" s="56"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="E21" s="64"/>
-      <c r="F21" s="66"/>
-      <c r="G21" s="66"/>
-      <c r="H21" s="66"/>
+      <c r="E21" s="56"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="57"/>
     </row>
     <row r="22" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A22" s="64"/>
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64" t="s">
+      <c r="A22" s="56"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="E22" s="64"/>
-      <c r="F22" s="66"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="66"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="57"/>
     </row>
     <row r="23" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A23" s="64"/>
-      <c r="B23" s="64"/>
-      <c r="C23" s="64"/>
-      <c r="D23" s="64" t="s">
+      <c r="A23" s="56"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="64"/>
-      <c r="F23" s="67" t="s">
+      <c r="E23" s="56"/>
+      <c r="F23" s="59" t="s">
         <v>81</v>
       </c>
-      <c r="G23" s="67"/>
-      <c r="H23" s="67"/>
+      <c r="G23" s="59"/>
+      <c r="H23" s="59"/>
     </row>
     <row r="24" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A24" s="64" t="s">
+      <c r="A24" s="56" t="s">
         <v>56</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -3900,7 +3885,7 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A25" s="64"/>
+      <c r="A25" s="56"/>
       <c r="B25" s="5" t="s">
         <v>61</v>
       </c>
@@ -3912,107 +3897,97 @@
       <c r="F25" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G25" s="66"/>
-      <c r="H25" s="66"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="57"/>
     </row>
     <row r="26" spans="1:8" ht="19.5" customHeight="1">
-      <c r="E26" s="72" t="s">
+      <c r="E26" s="58" t="s">
         <v>64</v>
       </c>
-      <c r="F26" s="72"/>
-      <c r="G26" s="72"/>
-      <c r="H26" s="72"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
     </row>
     <row r="27" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A27" s="64" t="s">
+      <c r="A27" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="B27" s="64"/>
-      <c r="C27" s="67" t="s">
+      <c r="B27" s="56"/>
+      <c r="C27" s="59" t="s">
         <v>74</v>
       </c>
-      <c r="D27" s="67"/>
-      <c r="E27" s="64" t="s">
+      <c r="D27" s="59"/>
+      <c r="E27" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="F27" s="64"/>
-      <c r="G27" s="66" t="s">
+      <c r="F27" s="56"/>
+      <c r="G27" s="57" t="s">
         <v>67</v>
       </c>
-      <c r="H27" s="66"/>
+      <c r="H27" s="57"/>
     </row>
     <row r="29" spans="1:8" ht="24" customHeight="1">
-      <c r="A29" s="70" t="s">
+      <c r="A29" s="54" t="s">
         <v>68</v>
       </c>
-      <c r="B29" s="70"/>
-      <c r="C29" s="70"/>
-      <c r="D29" s="70"/>
-      <c r="E29" s="70"/>
-      <c r="F29" s="70"/>
-      <c r="G29" s="70"/>
-      <c r="H29" s="70"/>
+      <c r="B29" s="54"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="54"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="54"/>
     </row>
     <row r="30" spans="1:8" ht="24" customHeight="1">
-      <c r="A30" s="70" t="s">
+      <c r="A30" s="54" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="70"/>
-      <c r="C30" s="70"/>
-      <c r="D30" s="70"/>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="70"/>
+      <c r="B30" s="54"/>
+      <c r="C30" s="54"/>
+      <c r="D30" s="54"/>
+      <c r="E30" s="54"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="54"/>
     </row>
     <row r="31" spans="1:8" ht="24" customHeight="1">
-      <c r="A31" s="70" t="s">
+      <c r="A31" s="54" t="s">
         <v>70</v>
       </c>
-      <c r="B31" s="70"/>
-      <c r="C31" s="70"/>
-      <c r="D31" s="70"/>
-      <c r="E31" s="70"/>
-      <c r="F31" s="70"/>
-      <c r="G31" s="70"/>
-      <c r="H31" s="70"/>
+      <c r="B31" s="54"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="54"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
+      <c r="H31" s="54"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="71" t="s">
+      <c r="A33" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="B33" s="71"/>
-      <c r="C33" s="71"/>
-      <c r="D33" s="71"/>
-      <c r="E33" s="71"/>
-      <c r="F33" s="71"/>
-      <c r="G33" s="71"/>
-      <c r="H33" s="71"/>
+      <c r="B33" s="55"/>
+      <c r="C33" s="55"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="55"/>
+      <c r="H33" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A33:H33"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="E26:H26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="G27:H27"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="D20:H20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:H21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:H22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A2:F3"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:H7"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:H8"/>
     <mergeCell ref="A9:B9"/>
@@ -4029,21 +4004,31 @@
     <mergeCell ref="D16:E19"/>
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="G17:H17"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="F6:H6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:H7"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A2:F3"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="D20:H20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="E26:H26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="G27:H27"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>